<commit_message>
Hibakezelés: todo E–J pontok javítása
- E: GEH_Main explicit result = ErrorAction.Continue
- F: analitikai idők Elapsed.TotalSeconds alapján (Seconds helyett)
- G: "utolsó kísérlet" döntés ErrorPolicy.IsLastAttempt-tel, új
  QueueMaxRetryNumber Config kulcs (RetryNo > 2 helyett)
- H: mellékletlista string.Join + File.Exists, DisplayName javítás
- I: SetTransactionStatus (Successful) és GetQueueItem mappa / queue név
  a Configból (Processes/Teszt, Teszt_queue beégetés megszűnt)
- J: Config betöltési hiba: FW-CFG-002 kód, Fatal log, tartalék e-mail
  az új in_FallbackAlertEmail Main argumentumra

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018Xr5LCgBZQ9r6MNW3GqXzJ
</commit_message>
<xml_diff>
--- a/Configuration/Config.xlsx
+++ b/Configuration/Config.xlsx
@@ -800,7 +800,7 @@
       <c r="B6" s="15" t="n"/>
       <c r="C6" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Az értéknek meg kell egyeznie az Orchestrator egyik mappájával, és ebben a mappában létre kell hozni egy OrchestratorQueueName nevű queuet. </t>
+          <t>Az értéknek meg kell egyeznie az Orchestrator egyik mappájával, és ebben a mappában létre kell hozni egy OrchestratorQueueName nevű queuet. Üresen hagyva a job saját Orchestrator mappáját használja.</t>
         </is>
       </c>
     </row>
@@ -808,6 +808,11 @@
       <c r="A7" s="12" t="inlineStr">
         <is>
           <t>OrchestratorQueueName</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Teszt_queue</t>
         </is>
       </c>
       <c r="C7" s="15" t="inlineStr">
@@ -1014,14 +1019,27 @@
       </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
-      <c r="A21" s="16" t="n"/>
-      <c r="B21" s="16" t="n"/>
-      <c r="C21" s="16" t="n"/>
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>QueueMaxRetryNumber</t>
+        </is>
+      </c>
+      <c r="B21" s="15" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C21" s="14" t="inlineStr">
+        <is>
+          <t>Meg kell egyeznie az Orchestrator queue "Max # Retries" beállításával. Ebből dönti el a keretrendszer, hogy egy rendszerhibás tétel az utolsó kísérletnél tart-e (ilyenkor fut a SystemExceptionHandling és megy ki a rendszerhiba e-mail). Üres / érvénytelen érték esetén minden kísérlet utolsónak számít.</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="A22" s="12" t="n"/>
       <c r="B22" s="13" t="n"/>
     </row>
+    <row r="23"/>
     <row r="24" ht="15" customHeight="1">
       <c r="A24" s="13" t="n"/>
     </row>

</xml_diff>